<commit_message>
update gen bench py
</commit_message>
<xml_diff>
--- a/templates/benchmark_beaters_template.xlsx
+++ b/templates/benchmark_beaters_template.xlsx
@@ -17,9 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Koyfin - US" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Cdn Hardcoded'!$A$1:$J$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Cdn Hardcoded'!$A$1:$J$60</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Cdn'!$A$1:$J$48</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'US Hardcoded'!$A$1:$J$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'US Hardcoded'!$A$1:$J$60</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'US'!$A$1:$J$54</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2124,7 +2124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.21875" customWidth="1" style="11" min="1" max="1"/>
@@ -2368,86 +2368,86 @@
     </row>
     <row r="16" ht="20.4" customHeight="1">
       <c r="A16" s="28" t="n"/>
-      <c r="B16" s="49" t="n"/>
-      <c r="C16" s="30" t="n"/>
-      <c r="D16" s="31" t="n"/>
-      <c r="E16" s="32" t="n"/>
-      <c r="F16" s="32" t="n"/>
+      <c r="B16" s="48" t="n"/>
+      <c r="C16" s="38" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="40" t="n"/>
+      <c r="F16" s="40" t="n"/>
       <c r="G16" s="89" t="n"/>
-      <c r="H16" s="91" t="n"/>
-      <c r="I16" s="54" t="n"/>
+      <c r="H16" s="90" t="n"/>
+      <c r="I16" s="53" t="n"/>
       <c r="J16" s="28" t="n"/>
     </row>
     <row r="17" ht="40.8" customHeight="1">
       <c r="A17" s="36" t="n"/>
-      <c r="B17" s="48" t="n"/>
-      <c r="C17" s="38" t="n"/>
-      <c r="D17" s="39" t="n"/>
-      <c r="E17" s="40" t="n"/>
-      <c r="F17" s="40" t="n"/>
+      <c r="B17" s="49" t="n"/>
+      <c r="C17" s="30" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="32" t="n"/>
+      <c r="F17" s="32" t="n"/>
       <c r="G17" s="89" t="n"/>
-      <c r="H17" s="90" t="n"/>
-      <c r="I17" s="53" t="n"/>
+      <c r="H17" s="91" t="n"/>
+      <c r="I17" s="54" t="n"/>
       <c r="J17" s="36" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="28" t="n"/>
-      <c r="B18" s="49" t="n"/>
-      <c r="C18" s="30" t="n"/>
-      <c r="D18" s="31" t="n"/>
-      <c r="E18" s="32" t="n"/>
-      <c r="F18" s="32" t="n"/>
+      <c r="B18" s="48" t="n"/>
+      <c r="C18" s="38" t="n"/>
+      <c r="D18" s="39" t="n"/>
+      <c r="E18" s="40" t="n"/>
+      <c r="F18" s="40" t="n"/>
       <c r="G18" s="89" t="n"/>
-      <c r="H18" s="91" t="n"/>
-      <c r="I18" s="54" t="n"/>
+      <c r="H18" s="90" t="n"/>
+      <c r="I18" s="53" t="n"/>
       <c r="J18" s="28" t="n"/>
     </row>
     <row r="19" ht="30.6" customHeight="1">
       <c r="A19" s="36" t="n"/>
-      <c r="B19" s="48" t="n"/>
-      <c r="C19" s="38" t="n"/>
-      <c r="D19" s="39" t="n"/>
-      <c r="E19" s="40" t="n"/>
-      <c r="F19" s="40" t="n"/>
+      <c r="B19" s="49" t="n"/>
+      <c r="C19" s="30" t="n"/>
+      <c r="D19" s="31" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
       <c r="G19" s="89" t="n"/>
-      <c r="H19" s="90" t="n"/>
-      <c r="I19" s="53" t="n"/>
+      <c r="H19" s="91" t="n"/>
+      <c r="I19" s="54" t="n"/>
       <c r="J19" s="36" t="n"/>
     </row>
     <row r="20" ht="30.6" customHeight="1">
       <c r="A20" s="28" t="n"/>
-      <c r="B20" s="49" t="n"/>
-      <c r="C20" s="30" t="n"/>
-      <c r="D20" s="31" t="n"/>
-      <c r="E20" s="32" t="n"/>
-      <c r="F20" s="32" t="n"/>
+      <c r="B20" s="48" t="n"/>
+      <c r="C20" s="38" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="40" t="n"/>
+      <c r="F20" s="40" t="n"/>
       <c r="G20" s="89" t="n"/>
-      <c r="H20" s="91" t="n"/>
-      <c r="I20" s="54" t="n"/>
+      <c r="H20" s="90" t="n"/>
+      <c r="I20" s="53" t="n"/>
       <c r="J20" s="28" t="n"/>
     </row>
     <row r="21" ht="30.6" customHeight="1">
       <c r="A21" s="36" t="n"/>
-      <c r="B21" s="48" t="n"/>
-      <c r="C21" s="38" t="n"/>
-      <c r="D21" s="39" t="n"/>
-      <c r="E21" s="40" t="n"/>
-      <c r="F21" s="40" t="n"/>
+      <c r="B21" s="49" t="n"/>
+      <c r="C21" s="30" t="n"/>
+      <c r="D21" s="31" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
       <c r="G21" s="89" t="n"/>
-      <c r="H21" s="90" t="n"/>
-      <c r="I21" s="53" t="n"/>
+      <c r="H21" s="91" t="n"/>
+      <c r="I21" s="54" t="n"/>
       <c r="J21" s="36" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="28" t="n"/>
-      <c r="B22" s="49" t="n"/>
-      <c r="C22" s="30" t="n"/>
-      <c r="D22" s="31" t="n"/>
-      <c r="E22" s="32" t="n"/>
-      <c r="F22" s="32" t="n"/>
+      <c r="B22" s="48" t="n"/>
+      <c r="C22" s="38" t="n"/>
+      <c r="D22" s="39" t="n"/>
+      <c r="E22" s="40" t="n"/>
+      <c r="F22" s="40" t="n"/>
       <c r="G22" s="89" t="n"/>
-      <c r="H22" s="91" t="n"/>
-      <c r="I22" s="54" t="n"/>
+      <c r="H22" s="90" t="n"/>
+      <c r="I22" s="53" t="n"/>
       <c r="J22" s="28" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
@@ -2500,38 +2500,38 @@
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="36" t="n"/>
-      <c r="B27" s="48" t="n"/>
-      <c r="C27" s="38" t="n"/>
-      <c r="D27" s="39" t="n"/>
-      <c r="E27" s="40" t="n"/>
-      <c r="F27" s="40" t="n"/>
+      <c r="B27" s="49" t="n"/>
+      <c r="C27" s="30" t="n"/>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="32" t="n"/>
       <c r="G27" s="89" t="n"/>
-      <c r="H27" s="90" t="n"/>
-      <c r="I27" s="53" t="n"/>
+      <c r="H27" s="91" t="n"/>
+      <c r="I27" s="54" t="n"/>
       <c r="J27" s="36" t="n"/>
     </row>
     <row r="28" ht="20.4" customHeight="1">
       <c r="A28" s="28" t="n"/>
-      <c r="B28" s="49" t="n"/>
-      <c r="C28" s="30" t="n"/>
-      <c r="D28" s="31" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="32" t="n"/>
+      <c r="B28" s="48" t="n"/>
+      <c r="C28" s="38" t="n"/>
+      <c r="D28" s="39" t="n"/>
+      <c r="E28" s="40" t="n"/>
+      <c r="F28" s="40" t="n"/>
       <c r="G28" s="89" t="n"/>
-      <c r="H28" s="91" t="n"/>
-      <c r="I28" s="54" t="n"/>
+      <c r="H28" s="90" t="n"/>
+      <c r="I28" s="53" t="n"/>
       <c r="J28" s="28" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="36" t="n"/>
-      <c r="B29" s="48" t="n"/>
-      <c r="C29" s="38" t="n"/>
-      <c r="D29" s="39" t="n"/>
-      <c r="E29" s="40" t="n"/>
-      <c r="F29" s="40" t="n"/>
+      <c r="B29" s="49" t="n"/>
+      <c r="C29" s="30" t="n"/>
+      <c r="D29" s="31" t="n"/>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="32" t="n"/>
       <c r="G29" s="89" t="n"/>
-      <c r="H29" s="90" t="n"/>
-      <c r="I29" s="53" t="n"/>
+      <c r="H29" s="91" t="n"/>
+      <c r="I29" s="54" t="n"/>
       <c r="J29" s="36" t="n"/>
     </row>
     <row r="30" ht="30.6" customHeight="1">
@@ -2668,118 +2668,228 @@
     </row>
     <row r="41" ht="15.6" customHeight="1" thickBot="1">
       <c r="A41" s="68" t="n"/>
-      <c r="B41" s="69" t="n"/>
-      <c r="C41" s="70" t="n"/>
-      <c r="D41" s="71" t="n"/>
-      <c r="E41" s="72" t="n"/>
-      <c r="F41" s="72" t="n"/>
-      <c r="G41" s="92" t="n"/>
-      <c r="H41" s="93" t="n"/>
-      <c r="I41" s="74" t="n"/>
+      <c r="B41" s="49" t="n"/>
+      <c r="C41" s="30" t="n"/>
+      <c r="D41" s="31" t="n"/>
+      <c r="E41" s="32" t="n"/>
+      <c r="F41" s="32" t="n"/>
+      <c r="G41" s="89" t="n"/>
+      <c r="H41" s="91" t="n"/>
+      <c r="I41" s="54" t="n"/>
       <c r="J41" s="68" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" ht="26.4" customHeight="1">
       <c r="A42" s="43" t="n"/>
-      <c r="B42" s="43" t="n"/>
-      <c r="C42" s="43" t="n"/>
-      <c r="D42" s="43" t="n"/>
-      <c r="E42" s="43" t="n"/>
-      <c r="F42" s="43" t="n"/>
-      <c r="G42" s="43" t="n"/>
-      <c r="H42" s="43" t="n"/>
-      <c r="I42" s="43" t="n"/>
+      <c r="B42" s="48" t="n"/>
+      <c r="C42" s="38" t="n"/>
+      <c r="D42" s="39" t="n"/>
+      <c r="E42" s="40" t="n"/>
+      <c r="F42" s="40" t="n"/>
+      <c r="G42" s="89" t="n"/>
+      <c r="H42" s="90" t="n"/>
+      <c r="I42" s="53" t="n"/>
       <c r="J42" s="43" t="n"/>
     </row>
-    <row r="43" ht="15.6" customHeight="1" thickBot="1">
+    <row r="43" ht="26.4" customHeight="1" thickBot="1">
       <c r="A43" s="43" t="n"/>
-      <c r="B43" s="43" t="n"/>
-      <c r="C43" s="43" t="n"/>
-      <c r="D43" s="43" t="n"/>
-      <c r="E43" s="43" t="n"/>
-      <c r="F43" s="43" t="n"/>
-      <c r="G43" s="43" t="n"/>
-      <c r="H43" s="43" t="n"/>
-      <c r="I43" s="43" t="n"/>
+      <c r="B43" s="49" t="n"/>
+      <c r="C43" s="30" t="n"/>
+      <c r="D43" s="31" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="89" t="n"/>
+      <c r="H43" s="91" t="n"/>
+      <c r="I43" s="54" t="n"/>
       <c r="J43" s="43" t="n"/>
     </row>
-    <row r="44" ht="12" customHeight="1">
+    <row r="44" ht="26.4" customHeight="1">
       <c r="A44" s="43" t="n"/>
-      <c r="B44" s="58" t="n"/>
-      <c r="C44" s="59" t="n"/>
-      <c r="D44" s="59" t="n"/>
-      <c r="E44" s="59" t="n"/>
-      <c r="F44" s="59" t="n"/>
-      <c r="G44" s="59" t="n"/>
-      <c r="H44" s="59" t="n"/>
-      <c r="I44" s="60" t="n"/>
+      <c r="B44" s="48" t="n"/>
+      <c r="C44" s="38" t="n"/>
+      <c r="D44" s="39" t="n"/>
+      <c r="E44" s="40" t="n"/>
+      <c r="F44" s="40" t="n"/>
+      <c r="G44" s="89" t="n"/>
+      <c r="H44" s="90" t="n"/>
+      <c r="I44" s="53" t="n"/>
       <c r="J44" s="43" t="n"/>
     </row>
-    <row r="45" ht="15.6" customHeight="1">
+    <row r="45" ht="26.4" customHeight="1">
       <c r="A45" s="43" t="n"/>
-      <c r="B45" s="67" t="n"/>
-      <c r="C45" s="64" t="n"/>
-      <c r="D45" s="66" t="n"/>
-      <c r="E45" s="64" t="n"/>
-      <c r="F45" s="64" t="n"/>
-      <c r="G45" s="64" t="n"/>
-      <c r="H45" s="64" t="n"/>
-      <c r="I45" s="65" t="n"/>
+      <c r="B45" s="49" t="n"/>
+      <c r="C45" s="30" t="n"/>
+      <c r="D45" s="31" t="n"/>
+      <c r="E45" s="32" t="n"/>
+      <c r="F45" s="32" t="n"/>
+      <c r="G45" s="89" t="n"/>
+      <c r="H45" s="91" t="n"/>
+      <c r="I45" s="54" t="n"/>
       <c r="J45" s="43" t="n"/>
     </row>
-    <row r="46" ht="9.6" customHeight="1" thickBot="1">
+    <row r="46" ht="26.4" customHeight="1" thickBot="1">
       <c r="A46" s="43" t="n"/>
-      <c r="B46" s="61" t="n"/>
-      <c r="C46" s="62" t="n"/>
-      <c r="D46" s="62" t="n"/>
-      <c r="E46" s="62" t="n"/>
-      <c r="F46" s="62" t="n"/>
-      <c r="G46" s="62" t="n"/>
-      <c r="H46" s="62" t="n"/>
-      <c r="I46" s="63" t="n"/>
+      <c r="B46" s="48" t="n"/>
+      <c r="C46" s="38" t="n"/>
+      <c r="D46" s="39" t="n"/>
+      <c r="E46" s="40" t="n"/>
+      <c r="F46" s="40" t="n"/>
+      <c r="G46" s="89" t="n"/>
+      <c r="H46" s="90" t="n"/>
+      <c r="I46" s="53" t="n"/>
       <c r="J46" s="43" t="n"/>
     </row>
-    <row r="47">
+    <row r="47" ht="26.4" customHeight="1">
       <c r="A47" s="43" t="n"/>
-      <c r="B47" s="43" t="n"/>
-      <c r="C47" s="43" t="n"/>
-      <c r="D47" s="43" t="n"/>
-      <c r="E47" s="43" t="n"/>
-      <c r="F47" s="43" t="n"/>
-      <c r="G47" s="43" t="n"/>
-      <c r="H47" s="43" t="n"/>
-      <c r="I47" s="43" t="n"/>
+      <c r="B47" s="49" t="n"/>
+      <c r="C47" s="30" t="n"/>
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="32" t="n"/>
+      <c r="F47" s="32" t="n"/>
+      <c r="G47" s="89" t="n"/>
+      <c r="H47" s="91" t="n"/>
+      <c r="I47" s="54" t="n"/>
       <c r="J47" s="43" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" ht="26.4" customHeight="1">
       <c r="A48" s="43" t="n"/>
-      <c r="B48" s="47" t="n"/>
-      <c r="C48" s="47" t="n"/>
-      <c r="D48" s="47" t="n"/>
-      <c r="E48" s="47" t="n"/>
-      <c r="F48" s="47" t="n"/>
-      <c r="G48" s="47" t="n"/>
-      <c r="H48" s="47" t="n"/>
-      <c r="I48" s="47" t="n"/>
+      <c r="B48" s="48" t="n"/>
+      <c r="C48" s="38" t="n"/>
+      <c r="D48" s="39" t="n"/>
+      <c r="E48" s="40" t="n"/>
+      <c r="F48" s="40" t="n"/>
+      <c r="G48" s="89" t="n"/>
+      <c r="H48" s="90" t="n"/>
+      <c r="I48" s="53" t="n"/>
       <c r="J48" s="43" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="26.4" customHeight="1">
       <c r="A49" s="43" t="n"/>
-      <c r="B49" s="43" t="n"/>
-      <c r="C49" s="43" t="n"/>
-      <c r="D49" s="43" t="n"/>
-      <c r="E49" s="43" t="n"/>
-      <c r="F49" s="43" t="n"/>
-      <c r="G49" s="43" t="n"/>
-      <c r="H49" s="43" t="n"/>
-      <c r="I49" s="43" t="n"/>
+      <c r="B49" s="49" t="n"/>
+      <c r="C49" s="30" t="n"/>
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="32" t="n"/>
+      <c r="F49" s="32" t="n"/>
+      <c r="G49" s="89" t="n"/>
+      <c r="H49" s="91" t="n"/>
+      <c r="I49" s="54" t="n"/>
       <c r="J49" s="43" t="n"/>
+    </row>
+    <row r="50" ht="26.4" customHeight="1">
+      <c r="B50" s="48" t="n"/>
+      <c r="C50" s="38" t="n"/>
+      <c r="D50" s="39" t="n"/>
+      <c r="E50" s="40" t="n"/>
+      <c r="F50" s="40" t="n"/>
+      <c r="G50" s="89" t="n"/>
+      <c r="H50" s="90" t="n"/>
+      <c r="I50" s="53" t="n"/>
+    </row>
+    <row r="51" ht="26.4" customHeight="1">
+      <c r="B51" s="49" t="n"/>
+      <c r="C51" s="30" t="n"/>
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="32" t="n"/>
+      <c r="F51" s="32" t="n"/>
+      <c r="G51" s="89" t="n"/>
+      <c r="H51" s="91" t="n"/>
+      <c r="I51" s="54" t="n"/>
+    </row>
+    <row r="52" ht="26.4" customHeight="1">
+      <c r="B52" s="48" t="n"/>
+      <c r="C52" s="38" t="n"/>
+      <c r="D52" s="39" t="n"/>
+      <c r="E52" s="40" t="n"/>
+      <c r="F52" s="40" t="n"/>
+      <c r="G52" s="89" t="n"/>
+      <c r="H52" s="90" t="n"/>
+      <c r="I52" s="53" t="n"/>
+    </row>
+    <row r="53" ht="26.4" customHeight="1">
+      <c r="B53" s="49" t="n"/>
+      <c r="C53" s="30" t="n"/>
+      <c r="D53" s="31" t="n"/>
+      <c r="E53" s="32" t="n"/>
+      <c r="F53" s="32" t="n"/>
+      <c r="G53" s="89" t="n"/>
+      <c r="H53" s="91" t="n"/>
+      <c r="I53" s="54" t="n"/>
+    </row>
+    <row r="54" ht="26.4" customHeight="1">
+      <c r="B54" s="48" t="n"/>
+      <c r="C54" s="38" t="n"/>
+      <c r="D54" s="39" t="n"/>
+      <c r="E54" s="40" t="n"/>
+      <c r="F54" s="40" t="n"/>
+      <c r="G54" s="89" t="n"/>
+      <c r="H54" s="90" t="n"/>
+      <c r="I54" s="53" t="n"/>
+    </row>
+    <row r="55" ht="26.4" customHeight="1">
+      <c r="B55" s="49" t="n"/>
+      <c r="C55" s="30" t="n"/>
+      <c r="D55" s="31" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="89" t="n"/>
+      <c r="H55" s="91" t="n"/>
+      <c r="I55" s="54" t="n"/>
+    </row>
+    <row r="56" ht="26.4" customHeight="1">
+      <c r="B56" s="48" t="n"/>
+      <c r="C56" s="38" t="n"/>
+      <c r="D56" s="39" t="n"/>
+      <c r="E56" s="40" t="n"/>
+      <c r="F56" s="40" t="n"/>
+      <c r="G56" s="89" t="n"/>
+      <c r="H56" s="90" t="n"/>
+      <c r="I56" s="53" t="n"/>
+    </row>
+    <row r="57" ht="26.4" customHeight="1">
+      <c r="B57" s="49" t="n"/>
+      <c r="C57" s="30" t="n"/>
+      <c r="D57" s="31" t="n"/>
+      <c r="E57" s="32" t="n"/>
+      <c r="F57" s="32" t="n"/>
+      <c r="G57" s="89" t="n"/>
+      <c r="H57" s="91" t="n"/>
+      <c r="I57" s="54" t="n"/>
+    </row>
+    <row r="58" ht="26.4" customHeight="1">
+      <c r="B58" s="48" t="n"/>
+      <c r="C58" s="38" t="n"/>
+      <c r="D58" s="39" t="n"/>
+      <c r="E58" s="40" t="n"/>
+      <c r="F58" s="40" t="n"/>
+      <c r="G58" s="89" t="n"/>
+      <c r="H58" s="90" t="n"/>
+      <c r="I58" s="53" t="n"/>
+    </row>
+    <row r="59" ht="26.4" customHeight="1">
+      <c r="B59" s="49" t="n"/>
+      <c r="C59" s="30" t="n"/>
+      <c r="D59" s="31" t="n"/>
+      <c r="E59" s="32" t="n"/>
+      <c r="F59" s="32" t="n"/>
+      <c r="G59" s="89" t="n"/>
+      <c r="H59" s="91" t="n"/>
+      <c r="I59" s="54" t="n"/>
+    </row>
+    <row r="60" ht="26.4" customHeight="1">
+      <c r="B60" s="48" t="n"/>
+      <c r="C60" s="38" t="n"/>
+      <c r="D60" s="39" t="n"/>
+      <c r="E60" s="40" t="n"/>
+      <c r="F60" s="40" t="n"/>
+      <c r="G60" s="89" t="n"/>
+      <c r="H60" s="90" t="n"/>
+      <c r="I60" s="53" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="H2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G8:G41">
+  <conditionalFormatting sqref="G8:G60">
     <cfRule type="colorScale" priority="1371">
       <colorScale>
         <cfvo type="min"/>
@@ -3644,7 +3754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I535"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -3694,540 +3804,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4254,7 +3830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.21875" customWidth="1" style="11" min="1" max="1"/>
@@ -4808,108 +4384,218 @@
       <c r="I41" s="54" t="n"/>
       <c r="J41" s="28" t="n"/>
     </row>
-    <row r="42" ht="24.6" customHeight="1" thickBot="1">
+    <row r="42" ht="24" customHeight="1" thickBot="1">
       <c r="A42" s="75" t="n"/>
-      <c r="B42" s="76" t="n"/>
-      <c r="C42" s="77" t="n"/>
-      <c r="D42" s="78" t="n"/>
-      <c r="E42" s="79" t="n"/>
-      <c r="F42" s="79" t="n"/>
-      <c r="G42" s="92" t="n"/>
-      <c r="H42" s="96" t="n"/>
-      <c r="I42" s="81" t="n"/>
+      <c r="B42" s="48" t="n"/>
+      <c r="C42" s="38" t="n"/>
+      <c r="D42" s="39" t="n"/>
+      <c r="E42" s="40" t="n"/>
+      <c r="F42" s="40" t="n"/>
+      <c r="G42" s="89" t="n"/>
+      <c r="H42" s="90" t="n"/>
+      <c r="I42" s="53" t="n"/>
       <c r="J42" s="75" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" ht="24" customHeight="1">
       <c r="A43" s="43" t="n"/>
-      <c r="B43" s="43" t="n"/>
-      <c r="C43" s="43" t="n"/>
-      <c r="D43" s="43" t="n"/>
-      <c r="E43" s="43" t="n"/>
-      <c r="F43" s="43" t="n"/>
-      <c r="G43" s="43" t="n"/>
-      <c r="H43" s="43" t="n"/>
-      <c r="I43" s="43" t="n"/>
+      <c r="B43" s="49" t="n"/>
+      <c r="C43" s="30" t="n"/>
+      <c r="D43" s="31" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="89" t="n"/>
+      <c r="H43" s="91" t="n"/>
+      <c r="I43" s="54" t="n"/>
       <c r="J43" s="43" t="n"/>
     </row>
-    <row r="44" ht="15.6" customHeight="1" thickBot="1">
+    <row r="44" ht="24" customHeight="1" thickBot="1">
       <c r="A44" s="43" t="n"/>
-      <c r="B44" s="43" t="n"/>
-      <c r="C44" s="43" t="n"/>
-      <c r="D44" s="43" t="n"/>
-      <c r="E44" s="43" t="n"/>
-      <c r="F44" s="43" t="n"/>
-      <c r="G44" s="43" t="n"/>
-      <c r="H44" s="43" t="n"/>
-      <c r="I44" s="43" t="n"/>
+      <c r="B44" s="48" t="n"/>
+      <c r="C44" s="38" t="n"/>
+      <c r="D44" s="39" t="n"/>
+      <c r="E44" s="40" t="n"/>
+      <c r="F44" s="40" t="n"/>
+      <c r="G44" s="89" t="n"/>
+      <c r="H44" s="90" t="n"/>
+      <c r="I44" s="53" t="n"/>
       <c r="J44" s="43" t="n"/>
     </row>
-    <row r="45" ht="10.2" customHeight="1">
+    <row r="45" ht="24" customHeight="1">
       <c r="A45" s="43" t="n"/>
-      <c r="B45" s="58" t="n"/>
-      <c r="C45" s="59" t="n"/>
-      <c r="D45" s="59" t="n"/>
-      <c r="E45" s="59" t="n"/>
-      <c r="F45" s="59" t="n"/>
-      <c r="G45" s="59" t="n"/>
-      <c r="H45" s="59" t="n"/>
-      <c r="I45" s="60" t="n"/>
+      <c r="B45" s="49" t="n"/>
+      <c r="C45" s="30" t="n"/>
+      <c r="D45" s="31" t="n"/>
+      <c r="E45" s="32" t="n"/>
+      <c r="F45" s="32" t="n"/>
+      <c r="G45" s="89" t="n"/>
+      <c r="H45" s="91" t="n"/>
+      <c r="I45" s="54" t="n"/>
       <c r="J45" s="43" t="n"/>
     </row>
-    <row r="46" ht="15.6" customHeight="1">
+    <row r="46" ht="24" customHeight="1">
       <c r="A46" s="43" t="n"/>
-      <c r="B46" s="67" t="n"/>
-      <c r="C46" s="64" t="n"/>
-      <c r="D46" s="64" t="n"/>
-      <c r="E46" s="64" t="n"/>
-      <c r="F46" s="64" t="n"/>
-      <c r="G46" s="64" t="n"/>
-      <c r="H46" s="64" t="n"/>
-      <c r="I46" s="65" t="n"/>
+      <c r="B46" s="48" t="n"/>
+      <c r="C46" s="38" t="n"/>
+      <c r="D46" s="39" t="n"/>
+      <c r="E46" s="40" t="n"/>
+      <c r="F46" s="40" t="n"/>
+      <c r="G46" s="89" t="n"/>
+      <c r="H46" s="90" t="n"/>
+      <c r="I46" s="53" t="n"/>
       <c r="J46" s="43" t="n"/>
     </row>
-    <row r="47" ht="10.8" customHeight="1" thickBot="1">
+    <row r="47" ht="24" customHeight="1" thickBot="1">
       <c r="A47" s="43" t="n"/>
-      <c r="B47" s="61" t="n"/>
-      <c r="C47" s="62" t="n"/>
-      <c r="D47" s="62" t="n"/>
-      <c r="E47" s="62" t="n"/>
-      <c r="F47" s="62" t="n"/>
-      <c r="G47" s="62" t="n"/>
-      <c r="H47" s="62" t="n"/>
-      <c r="I47" s="63" t="n"/>
+      <c r="B47" s="49" t="n"/>
+      <c r="C47" s="30" t="n"/>
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="32" t="n"/>
+      <c r="F47" s="32" t="n"/>
+      <c r="G47" s="89" t="n"/>
+      <c r="H47" s="91" t="n"/>
+      <c r="I47" s="54" t="n"/>
       <c r="J47" s="43" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" ht="24" customHeight="1">
       <c r="A48" s="43" t="n"/>
-      <c r="B48" s="43" t="n"/>
-      <c r="C48" s="43" t="n"/>
-      <c r="D48" s="43" t="n"/>
-      <c r="E48" s="43" t="n"/>
-      <c r="F48" s="43" t="n"/>
-      <c r="G48" s="43" t="n"/>
-      <c r="H48" s="43" t="n"/>
-      <c r="I48" s="43" t="n"/>
+      <c r="B48" s="48" t="n"/>
+      <c r="C48" s="38" t="n"/>
+      <c r="D48" s="39" t="n"/>
+      <c r="E48" s="40" t="n"/>
+      <c r="F48" s="40" t="n"/>
+      <c r="G48" s="89" t="n"/>
+      <c r="H48" s="90" t="n"/>
+      <c r="I48" s="53" t="n"/>
       <c r="J48" s="43" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="24" customHeight="1">
       <c r="A49" s="43" t="n"/>
-      <c r="B49" s="47" t="n"/>
-      <c r="C49" s="47" t="n"/>
-      <c r="D49" s="47" t="n"/>
-      <c r="E49" s="47" t="n"/>
-      <c r="F49" s="47" t="n"/>
-      <c r="G49" s="47" t="n"/>
-      <c r="H49" s="47" t="n"/>
-      <c r="I49" s="47" t="n"/>
+      <c r="B49" s="49" t="n"/>
+      <c r="C49" s="30" t="n"/>
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="32" t="n"/>
+      <c r="F49" s="32" t="n"/>
+      <c r="G49" s="89" t="n"/>
+      <c r="H49" s="91" t="n"/>
+      <c r="I49" s="54" t="n"/>
       <c r="J49" s="43" t="n"/>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="B50" s="48" t="n"/>
+      <c r="C50" s="38" t="n"/>
+      <c r="D50" s="39" t="n"/>
+      <c r="E50" s="40" t="n"/>
+      <c r="F50" s="40" t="n"/>
+      <c r="G50" s="89" t="n"/>
+      <c r="H50" s="90" t="n"/>
+      <c r="I50" s="53" t="n"/>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="B51" s="49" t="n"/>
+      <c r="C51" s="30" t="n"/>
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="32" t="n"/>
+      <c r="F51" s="32" t="n"/>
+      <c r="G51" s="89" t="n"/>
+      <c r="H51" s="91" t="n"/>
+      <c r="I51" s="54" t="n"/>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="B52" s="48" t="n"/>
+      <c r="C52" s="38" t="n"/>
+      <c r="D52" s="39" t="n"/>
+      <c r="E52" s="40" t="n"/>
+      <c r="F52" s="40" t="n"/>
+      <c r="G52" s="89" t="n"/>
+      <c r="H52" s="90" t="n"/>
+      <c r="I52" s="53" t="n"/>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="B53" s="49" t="n"/>
+      <c r="C53" s="30" t="n"/>
+      <c r="D53" s="31" t="n"/>
+      <c r="E53" s="32" t="n"/>
+      <c r="F53" s="32" t="n"/>
+      <c r="G53" s="89" t="n"/>
+      <c r="H53" s="91" t="n"/>
+      <c r="I53" s="54" t="n"/>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="B54" s="48" t="n"/>
+      <c r="C54" s="38" t="n"/>
+      <c r="D54" s="39" t="n"/>
+      <c r="E54" s="40" t="n"/>
+      <c r="F54" s="40" t="n"/>
+      <c r="G54" s="89" t="n"/>
+      <c r="H54" s="90" t="n"/>
+      <c r="I54" s="53" t="n"/>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="B55" s="49" t="n"/>
+      <c r="C55" s="30" t="n"/>
+      <c r="D55" s="31" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="89" t="n"/>
+      <c r="H55" s="91" t="n"/>
+      <c r="I55" s="54" t="n"/>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="B56" s="48" t="n"/>
+      <c r="C56" s="38" t="n"/>
+      <c r="D56" s="39" t="n"/>
+      <c r="E56" s="40" t="n"/>
+      <c r="F56" s="40" t="n"/>
+      <c r="G56" s="89" t="n"/>
+      <c r="H56" s="90" t="n"/>
+      <c r="I56" s="53" t="n"/>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="B57" s="49" t="n"/>
+      <c r="C57" s="30" t="n"/>
+      <c r="D57" s="31" t="n"/>
+      <c r="E57" s="32" t="n"/>
+      <c r="F57" s="32" t="n"/>
+      <c r="G57" s="89" t="n"/>
+      <c r="H57" s="91" t="n"/>
+      <c r="I57" s="54" t="n"/>
+    </row>
+    <row r="58" ht="24" customHeight="1">
+      <c r="B58" s="48" t="n"/>
+      <c r="C58" s="38" t="n"/>
+      <c r="D58" s="39" t="n"/>
+      <c r="E58" s="40" t="n"/>
+      <c r="F58" s="40" t="n"/>
+      <c r="G58" s="89" t="n"/>
+      <c r="H58" s="90" t="n"/>
+      <c r="I58" s="53" t="n"/>
+    </row>
+    <row r="59" ht="24" customHeight="1">
+      <c r="B59" s="49" t="n"/>
+      <c r="C59" s="30" t="n"/>
+      <c r="D59" s="31" t="n"/>
+      <c r="E59" s="32" t="n"/>
+      <c r="F59" s="32" t="n"/>
+      <c r="G59" s="89" t="n"/>
+      <c r="H59" s="91" t="n"/>
+      <c r="I59" s="54" t="n"/>
+    </row>
+    <row r="60" ht="24" customHeight="1">
+      <c r="B60" s="48" t="n"/>
+      <c r="C60" s="38" t="n"/>
+      <c r="D60" s="39" t="n"/>
+      <c r="E60" s="40" t="n"/>
+      <c r="F60" s="40" t="n"/>
+      <c r="G60" s="89" t="n"/>
+      <c r="H60" s="90" t="n"/>
+      <c r="I60" s="53" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="H2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G8:G42">
+  <conditionalFormatting sqref="G8:G60">
     <cfRule type="colorScale" priority="1351">
       <colorScale>
         <cfvo type="min"/>
@@ -5774,7 +5460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I500"/>
+  <dimension ref="A1:I415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -5824,509 +5510,12 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
     <row r="112" ht="409.6" customHeight="1">
       <c r="I112" s="56" t="n"/>
     </row>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
     <row r="415" ht="409.6" customHeight="1">
       <c r="I415" s="56" t="n"/>
     </row>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>